<commit_message>
Update serializer and insurance calculator.
</commit_message>
<xml_diff>
--- a/insurance_calculator_project/insurance_calculator_app/tests/calculator_tests/expected_tariffs_files/different_cases/cumulative_insurance_annually_tariffs.xlsx
+++ b/insurance_calculator_project/insurance_calculator_app/tests/calculator_tests/expected_tariffs_files/different_cases/cumulative_insurance_annually_tariffs.xlsx
@@ -551,7 +551,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tariffs table in % with insurance premium rate 5.00% and loading 20.00%</t>
+          <t>Tariffs table in % with technical interest rate 5.00% and loading 20.00%</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Payment frequency: annually</t>
+          <t>Insurance premium payment frequency: annually</t>
         </is>
       </c>
     </row>

</xml_diff>